<commit_message>
Phase 1 fixes: shared export, odometer autofill, error handling
- Unify XLSX/CSV export into src/shared/exportWorkbook.ts; fixes
  desktop SUM formula that skipped the last data row
- Add UTF-8 BOM and CRLF to CSV so Czech diacritics open correctly
  in Excel
- Stop silently rewriting odometers on load/save/export; fill missing
  odometer start from the previous trip on save instead, and add an
  explicit confirmed "Recalculate odometers" button in Settings
- Add vehicle and driver filters to the trips list
- Handle localStorage quota errors and IPC failures with user-facing
  messages
- Remove default password hint from the login screen
- Stop dropping inferred drivers beyond three when loading legacy JSON
- Remove duplicated renderer types.ts in favour of src/shared/types.ts
- Move @vitejs/plugin-react to devDependencies

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-data/ukazkovy-export.xlsx
+++ b/sample-data/ukazkovy-export.xlsx
@@ -206,7 +206,7 @@
     <t>2026</t>
   </si>
   <si>
-    <t>7. 6. 2026 23:14:25</t>
+    <t>12. 6. 2026 13:21:15</t>
   </si>
   <si>
     <t>Značka</t>
@@ -899,7 +899,7 @@
         <v>44</v>
       </c>
       <c r="M6" s="5">
-        <f>SUM(M2:M4)</f>
+        <f>SUM(M2:M5)</f>
       </c>
     </row>
   </sheetData>
@@ -1017,7 +1017,7 @@
         <v>44</v>
       </c>
       <c r="G4" s="5">
-        <f>SUM(G2:G2)</f>
+        <f>SUM(G2:G3)</f>
       </c>
     </row>
   </sheetData>

</xml_diff>